<commit_message>
Actualización general de Documentación
</commit_message>
<xml_diff>
--- a/Fase 2/Evidencias Proyecto/Evidencias de Documentación/Carta Gantt CuTuCo.xlsx
+++ b/Fase 2/Evidencias Proyecto/Evidencias de Documentación/Carta Gantt CuTuCo.xlsx
@@ -163,13 +163,13 @@
     <t>Ajuste de requerimientos al alcance actualizado (Queda / No queda)</t>
   </si>
   <si>
-    <t>Modelo de datos: DER, tablas productores (rut_oficial, codigo_comercio_mall) y payments, RLS y policies</t>
-  </si>
-  <si>
-    <t>Arquitectura: Supabase (GoTrue, PostgREST), FastAPI y despliegue</t>
-  </si>
-  <si>
-    <t>Mockups de interfaz Vue.js (cliente, productor y administración)</t>
+    <t>Modelo de datos: MER, tablas productores (rut_oficial, codigo_comercio_mall) y payments, RLS y policies</t>
+  </si>
+  <si>
+    <t>Arquitectura: Supabase (GoTrue, PostgREST), FastAPI solo para Webpay y despliegue</t>
+  </si>
+  <si>
+    <t>Mockups de interfaz Vue.js (cliente, productor, administración y reclamos)</t>
   </si>
   <si>
     <t>Plan de Calidad y de Costos</t>
@@ -190,16 +190,16 @@
     <t>Migración SQLite a PostgreSQL y scripts de creación (DDL)</t>
   </si>
   <si>
-    <t>Autenticación y roles con GoTrue; bloqueo tras 5 intentos (FastAPI)</t>
-  </si>
-  <si>
-    <t>Registro de cliente y productor; aprobación de productores con Código de Comercio Mall</t>
+    <t>Autenticación, roles y permisos con GoTrue, RLS y policies (Supabase Auth)</t>
+  </si>
+  <si>
+    <t>Registro de cliente y productor; aprobación de postulaciones y registro del Código de Comercio Mall</t>
   </si>
   <si>
     <t>Catálogo con acceso invitado, buscador y carrito (Vue.js)</t>
   </si>
   <si>
-    <t>Consultas por PostgREST: productos, pedidos, usuarios y categorías</t>
+    <t>Consultas por PostgREST: productos, pedidos, usuarios, categorías y reclamos</t>
   </si>
   <si>
     <t>Panel del productor: productos, stock y ventas</t>
@@ -211,22 +211,22 @@
     <t>Pago con Webpay Mall (Split Payment: create, token_ws, commit) e idempotencia</t>
   </si>
   <si>
-    <t>Liquidación directa por pasarela (Split Payment) y reembolsos</t>
-  </si>
-  <si>
-    <t>Checkout y seguimiento del pedido (Vue.js)</t>
-  </si>
-  <si>
-    <t>Panel de administración y dashboard (aprobaciones, sanciones, pagos)</t>
+    <t>Gestión de reclamos (RF-027): registro, seguimiento, resolución y apelaciones</t>
+  </si>
+  <si>
+    <t>Checkout, seguimiento del pedido y registro de reclamos (Vue.js)</t>
+  </si>
+  <si>
+    <t>Panel de administración y dashboard (aprobaciones, reclamos, sanciones y pagos)</t>
   </si>
   <si>
     <t>Entrega con código de verificación (Preparación, En Tránsito, Entregado)</t>
   </si>
   <si>
-    <t>Calificaciones de 1 a 5, promedio y sanciones manuales</t>
-  </si>
-  <si>
-    <t>Correos con Resend (Auth por SMTP de Supabase y notificaciones)</t>
+    <t>Calificaciones de 1 a 5, promedio, sanciones manuales y apelaciones</t>
+  </si>
+  <si>
+    <t>Correos con Resend (autenticación por el SMTP de Supabase, detalle de compra y aviso de nuevo pedido)</t>
   </si>
   <si>
     <t>Validaciones: Vuelidate en frontend y Pydantic/constraints en backend</t>
@@ -250,7 +250,7 @@
     <t>Pruebas de integración de la API REST</t>
   </si>
   <si>
-    <t>Pruebas E2E de flujos críticos (compra, pago, entrega, calificación)</t>
+    <t>Pruebas E2E de flujos críticos (compra, pago, entrega, calificación y reclamo)</t>
   </si>
   <si>
     <t>Corrección de defectos y regresión</t>
@@ -337,7 +337,7 @@
     <t>2.1 ERS, criterios de aceptación y ajuste de requerimientos (Queda / No queda)</t>
   </si>
   <si>
-    <t>2.2 / 2.3 Modelo de datos (DER, productores, payments, RLS) y arquitectura de la solución</t>
+    <t>2.2 / 2.3 Modelo de datos (MER, productores, payments, RLS) y arquitectura de la solución</t>
   </si>
   <si>
     <t>2.4 Mockups Vue.js: cliente, productor, administración, checkout y entrega</t>
@@ -358,13 +358,13 @@
     <t>3.3 / 4.2 / 4.3 Catálogo invitado, carrito, registro, panel productor y CRUD base (PostgREST)</t>
   </si>
   <si>
-    <t>3.4 / 4.5 Webpay Mall (Split Payment), liquidación por pasarela, reembolsos y checkout</t>
-  </si>
-  <si>
-    <t>3.5 / 3.6 / 4.4 Entrega con código, venta por región, calificaciones, sanciones y correos</t>
-  </si>
-  <si>
-    <t>4.4 / 4.6 / 6.1 Dashboard admin, validaciones (Vuelidate) y pruebas unitarias</t>
+    <t>3.4 / 4.5 Webpay Mall (Split Payment), dispersión por pasarela y checkout</t>
+  </si>
+  <si>
+    <t>3.5 / 3.6 / 4.4 Entrega con código, venta por región, calificaciones, reclamos (RF-027), sanciones y correos</t>
+  </si>
+  <si>
+    <t>4.4 / 4.6 / 6.1 Dashboard admin (reclamos y sanciones), validaciones (Vuelidate) y pruebas unitarias</t>
   </si>
   <si>
     <t>COSTO HH POR ROL</t>
@@ -409,10 +409,10 @@
     <t>El costo por hora usa sueldos referenciales (hoja Analisis de Ingresos); no son pagos reales del proyecto.</t>
   </si>
   <si>
-    <t>Alcance actualizado: no planificamos historial de precios, stock bajo, múltiples admins, retención de carnet ni rate limiting.</t>
-  </si>
-  <si>
-    <t>Sin geolocalización, fotos obligatorias ni cosecha del día: la entrega se confirma con código y las sanciones son manuales.</t>
+    <t>Alcance actualizado: no planificamos historial de precios, avisos de stock bajo, múltiples administradores ni rate limiting propio, y RF-015 (almacenamiento de datos sensibles, como el carnet de identidad) queda eliminado.</t>
+  </si>
+  <si>
+    <t>Sin geolocalización, fotos obligatorias ni cosecha del día: la entrega se confirma con código, la validación de palabras prohibidas es automática por triggers y las sanciones son manuales, con reclamos y apelaciones (RF-027).</t>
   </si>
   <si>
     <t>Correspondencia entre los bloques de la EDT (6 bloques, 34 paquetes) y las 4 fases del proyecto (Acta de Constitución):</t>

</xml_diff>